<commit_message>
feat: add subcategory management drawer, category/test forms, and bulk import templates
</commit_message>
<xml_diff>
--- a/public/templates/1_Litmus_Categories_Bulk_Template.xlsx
+++ b/public/templates/1_Litmus_Categories_Bulk_Template.xlsx
@@ -488,18 +488,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="86" customWidth="1" min="1" max="1"/>
-    <col width="117" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="111" customWidth="1" min="1" max="1"/>
+    <col width="93" customWidth="1" min="2" max="2"/>
+    <col width="117" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>INSTRUCTIONS: Fill Category names and descriptions. Category names must be unique.</t>
+          <t>INSTRUCTIONS: Fill Category names, optional subcategories, and descriptions. Category names must be unique.</t>
         </is>
       </c>
     </row>
@@ -511,10 +512,15 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>subcategories</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>imageUrl</t>
         </is>
@@ -536,6 +542,11 @@
           <t>OPTIONAL</t>
         </is>
       </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -545,10 +556,15 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
+          <t>Raw Milk, Pasteurized Milk, Cheese &amp; Paneer, Butter &amp; Ghee, Yogurt &amp; Curd, Ice Cream</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
           <t>Safety, quality, and nutritional analysis for raw milk, pasteurized milk, cheese, butter, paneer, and ice creams.</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>https://example.com/images/dairy.png</t>
         </is>
@@ -562,10 +578,15 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
+          <t>Packaged Drinking Water, Carbonated Beverages, Fruit Juices &amp; Squashes, Tea &amp; Coffee</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
           <t>Physicochemical and microbial profiling for packaged water, fruit juices, carbonated drinks, tea, and coffee.</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -575,10 +596,15 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
+          <t>Bread &amp; Buns, Biscuits &amp; Cookies, Cakes &amp; Pastries, Chocolates &amp; Candies</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
           <t>Testing for flour quality, moisture, preservatives, sugar profile, and shelf-life analysis for baked goods.</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -588,10 +614,15 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
+          <t>Fresh Raw Meat, Processed Meat &amp; Sausages, Poultry &amp; Eggs, Fish &amp; Shellfish</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
           <t>Veterinary drug residue, heavy metals, microbial safety (Salmonella, Listeria), and freshness parameters.</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -601,14 +632,19 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
+          <t>Edible Vegetable Oils, Hydrogenated Fats (Vanaspati), Olive &amp; Specialty Oils, Animal Fats</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
           <t>Fatty acid profiling, Rancidity, Peroxide value, Free Fatty Acids (FFA), and adulteration screening.</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr"/>
+      <c r="D8" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>